<commit_message>
docs: export approved Xuanjia and Shanhe sets
</commit_message>
<xml_diff>
--- a/docs/design/2026-09-04-project-design-tables/GameXXK_装备设计总表_2026-09-04.xlsx
+++ b/docs/design/2026-09-04-project-design-tables/GameXXK_装备设计总表_2026-09-04.xlsx
@@ -13,10 +13,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_装备模板" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_词缀目录" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_套装效果" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_至宝配装基准" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_掉落等级带" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_实现差异" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_来源校验" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05A_套装术语" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_至宝配装基准" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_掉落等级带" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_实现差异" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_来源校验" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_说明'!$A$1:$B$9</definedName>
@@ -25,10 +26,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_装备模板'!$A$1:$H$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_词缀目录'!$A$1:$I$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_套装效果'!$A$1:$G$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_至宝配装基准'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_掉落等级带'!$A$1:$F$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_实现差异'!$A$1:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_来源校验'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'05A_套装术语'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'06_至宝配装基准'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'07_掉落等级带'!$A$1:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'08_实现差异'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'09_来源校验'!$A$1:$B$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -642,7 +644,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>当前运行时代码仍是旧曲线/旧宝石规则；本表是批准设计，不冒充已实装</t>
+          <t>装备基础曲线/宝石仍按差异表追踪；六套2／4／6件效果已实装，玄甲/山河采用v35语义</t>
         </is>
       </c>
     </row>
@@ -658,7 +660,204 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>当前旧实现</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>批准新设计</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>装备基础贡献</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>当前代码使用旧完整曲线</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>新设计生命/攻击/防御贡献约减半</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>宝石生命</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>当前代码为同阶攻防的10倍</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>新设计为5倍</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>不朽后成长</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>当前代码继续×2</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>新设计约×1.25并向上取整</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>待实现</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>至宝孔位</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>当前代码按品质公式得到2孔</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>新设计至宝整套共12孔，即每件2孔</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>装备内力</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>旧ID/快照仍可读</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>有效贡献恒为0</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>基础规则已冻结</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>玄甲/山河套装</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>旧描述符缺少完整消费者</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>六档批准语义与触发顺序</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>已实装并迁移至v35</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>百级最终属性</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>旧运行时投影不同</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>使用01表批准数值</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>设计冻结、运行时待迁移</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D8"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -692,17 +891,41 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>docs\superpowers\specs\2026-09-04-xuanjia-shanhe-set-design.md</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>20fd4db40aaa3fba6113c0975113c93192a85a76d3a7dcb2cf459f24499ce208</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
           <t>Source\GameXXK\Private\GameXXKEquipmentCatalog.cpp</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>767776be3c0d6809e9f5eac782270ca8a984743a0cd2027da5d06f48ad5a8f46</t>
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Source\GameXXK\Private\GameXXKEquipmentSetCatalog.cpp</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>f1137fa7394b30778a9b9a35bd6e0c798adca328896e9d2b3900743a67e77f80</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B3"/>
+  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6212,17 +6435,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>被动</t>
+          <t>产生护甲</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>获得的护甲提高5%。</t>
+          <t>穿戴者产生的护甲提高10%。</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>仅描述符；玄甲现行目标与阶位待评审</t>
+          <t>已批准；消费者已实装</t>
         </is>
       </c>
     </row>
@@ -6247,17 +6470,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>回合开始</t>
+          <t>回合开始／首次格挡</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>回合开始保留护甲并使首次直接受击反击80%。</t>
+          <t>我方回合开始时保留50%护甲；每个敌方回合首次格挡后，追加80%攻击伤害。</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>仅描述符；已确认意图为保留50%护甲，阶位/取整待评审</t>
+          <t>已批准；消费者已实装</t>
         </is>
       </c>
     </row>
@@ -6277,22 +6500,22 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>全队</t>
+          <t>全队唯一</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>首次友方生命受伤</t>
+          <t>首次攻击气血伤害</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>每回合首次有友方受到气血伤害时，为全队提供1次护甲与护援。</t>
+          <t>全队唯一。敌方回合首次有友方因攻击损失气血后，全体获得穿戴者40%防御的护甲；穿戴者援护其他友方各1次。</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>仅描述符；无战斗消费者</t>
+          <t>已批准；消费者已实装</t>
         </is>
       </c>
     </row>
@@ -6632,17 +6855,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>被动</t>
+          <t>首张地势牌</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>当前地形效果提高5%。</t>
+          <t>每回合首次打出地势牌后，抽1张。</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>仅描述符；待评审</t>
+          <t>已批准；消费者已实装</t>
         </is>
       </c>
     </row>
@@ -6667,17 +6890,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>首张地形联动牌</t>
+          <t>首张地势牌</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>费用降低1并强化相邻队友。</t>
+          <t>每回合首张地势牌少耗1气；结算后，其他友方各回复2内力。</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>仅描述符；相邻/增益/取整待评审</t>
+          <t>已批准；消费者已实装</t>
         </is>
       </c>
     </row>
@@ -6697,22 +6920,22 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>全队</t>
+          <t>全队唯一</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>被动</t>
+          <t>我方回合开始</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>当前地形成为阵眼，向全队提供12%对应增益。</t>
+          <t>全队唯一。每个我方回合开始时，由穿戴者触发1次当前地势。</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>仅描述符；无战斗消费者</t>
+          <t>已批准；消费者已实装</t>
         </is>
       </c>
     </row>
@@ -6723,6 +6946,61 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>术语</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>玩家说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>地势牌</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>会改变或触发地势的主动牌。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>全队唯一</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>同名团队套装只生效1份。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6896,7 +7174,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7597,179 +7875,4 @@
   <autoFilter ref="A1:F28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>项目</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>当前旧实现</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>批准新设计</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>状态</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>装备基础贡献</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>当前代码使用旧完整曲线</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>新设计生命/攻击/防御贡献约减半</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>待实现</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>宝石生命</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>当前代码为同阶攻防的10倍</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>新设计为5倍</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>待实现</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>不朽后成长</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>当前代码继续×2</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>新设计约×1.25并向上取整</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>待实现</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>至宝孔位</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>当前代码按品质公式得到2孔</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>新设计至宝整套共12孔，即每件2孔</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>一致</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>装备内力</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>旧ID/快照仍可读</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>有效贡献恒为0</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>基础规则已冻结</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>百级最终属性</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>旧运行时投影不同</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>使用01表批准数值</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>设计冻结、运行时待迁移</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:D7"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>